<commit_message>
add break logic and generate_break function
</commit_message>
<xml_diff>
--- a/shift_test2.xlsx
+++ b/shift_test2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\24y1034\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\24y1034\Desktop\BaristaBoard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56E25342-53E7-4110-B02A-5D745F580746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C2C9BB2-87F4-4031-98D1-CBFBF618793F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7680" yWindow="3020" windowWidth="11520" windowHeight="8260" xr2:uid="{03851545-BBB4-476B-A1CC-63F511BBC163}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{03851545-BBB4-476B-A1CC-63F511BBC163}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>